<commit_message>
Fix More Issue Names with Samples
</commit_message>
<xml_diff>
--- a/embeddings/sandbox/blender/plots/df_all_pca_donut.xlsx
+++ b/embeddings/sandbox/blender/plots/df_all_pca_donut.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="real" sheetId="1" state="visible" r:id="rId2"/>
@@ -952,10 +952,10 @@
     <t xml:space="preserve">es-digital-line-degradation-seq_spanish_liceo_0616_0</t>
   </si>
   <si>
-    <t xml:space="preserve">es-digital-line-degradation-seq_spanish_liceo_0616_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">es-digital-line-degradation-seq_spanish_liceo_0616_2</t>
+    <t xml:space="preserve">es-digital-line-degradation-seq_spanish_patria_0174_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">es-digital-line-degradation-seq_spanish_liceo_0282_2</t>
   </si>
   <si>
     <t xml:space="preserve">es-digital-line-degradation-seq_spanish_liceo_0384_1</t>
@@ -5493,6 +5493,9 @@
   </sheetPr>
   <dimension ref="A1:D152"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34.79"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -7641,7 +7644,7 @@
   <dimension ref="A1:AI280"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="54.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9921,6 +9924,9 @@
   </sheetPr>
   <dimension ref="A1:D152"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="53.47"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -16362,6 +16368,9 @@
   </sheetPr>
   <dimension ref="A1:D152"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50.92"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>